<commit_message>
fix bet side colors and update salary cap data
</commit_message>
<xml_diff>
--- a/data/raw_data/salary_cap/salary_cap_raw.xlsx
+++ b/data/raw_data/salary_cap/salary_cap_raw.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cuny620-my.sharepoint.com/personal/david_nemirovsky71_myhunter_cuny_edu/Documents/Documents/Football-DNA/data/raw_data/salary_cap/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive - Hunter - CUNY\Documents\Football-DNA\data\raw_data\salary_cap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{FDC5F9F0-9DC4-4C59-A899-7B05E0C72E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF4A8348-1236-462B-9EE7-33C164F796F1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0331370-AAFF-4A92-A38D-966F1428D7CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3E229123-87C5-4997-BE69-F48200F9557E}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="132">
   <si>
     <t>Cleveland Browns</t>
   </si>
@@ -563,6 +563,113 @@
     <t>TRENDING PLAYERS</t>
   </si>
   <si>
+    <t>TRENDING PAGES</t>
+  </si>
+  <si>
+    <t>Record</t>
+  </si>
+  <si>
+    <r>
+      <t>Players</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="4"/>
+        <color rgb="FF373F50"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>Active</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Age</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="4"/>
+        <color rgb="FF373F50"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>Average</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Total Cap</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="4"/>
+        <color rgb="FF373F50"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>Allocations</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Cap Space</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="4"/>
+        <color rgb="FF373F50"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>All</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Active</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="4"/>
+        <color rgb="FF373F50"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>53-Man</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Reserves</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="4"/>
+        <color rgb="FF373F50"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>IR/PUP/NFI/SUSP</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Dead</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="4"/>
+        <color rgb="FF373F50"/>
+        <rFont val="Roboto"/>
+      </rPr>
+      <t>Cap</t>
+    </r>
+  </si>
+  <si>
+    <t>- </t>
+  </si>
+  <si>
     <r>
       <t>1</t>
     </r>
@@ -570,19 +677,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Deshaun Watson </t>
+      <t> Aaron Donald </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(QB, CLE)</t>
+      <t>(DT, LAR)</t>
     </r>
   </si>
   <si>
@@ -593,19 +698,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Josh Jacobs </t>
+      <t> Joe Milton III </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(RB, GB)</t>
+      <t>(QB, DAL)</t>
     </r>
   </si>
   <si>
@@ -616,19 +719,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Leonard Williams </t>
+      <t> Kyler Gordon </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(DE, SEA)</t>
+      <t>(CB, CHI)</t>
     </r>
   </si>
   <si>
@@ -639,19 +740,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Lamar Jackson </t>
+      <t> Tua Tagovailoa </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(QB, BAL)</t>
+      <t>(QB, ATL)</t>
     </r>
   </si>
   <si>
@@ -662,19 +761,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> D.K. Metcalf </t>
+      <t> Odell Beckham, Jr. </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(WR, PIT)</t>
+      <t>(WR, NYG)</t>
     </r>
   </si>
   <si>
@@ -685,19 +782,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Kirk Cousins </t>
+      <t> Myles Garrett </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(QB, LV)</t>
+      <t>(OLB, LAR)</t>
     </r>
   </si>
   <si>
@@ -708,19 +803,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> TuTu Atwell </t>
+      <t> Will Levis </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(WR, LAR)</t>
+      <t>(QB, TEN)</t>
     </r>
   </si>
   <si>
@@ -731,19 +824,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Christian Gonzalez </t>
+      <t> Josh Jacobs </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(CB, NE)</t>
+      <t>(RB, GB)</t>
     </r>
   </si>
   <si>
@@ -754,19 +845,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Tua Tagovailoa </t>
+      <t> Deshaun Watson </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(QB, ATL)</t>
+      <t>(QB, CLE)</t>
     </r>
   </si>
   <si>
@@ -777,19 +866,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Patrick Mahomes </t>
+      <t> Phillip Buchanon </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(QB, KC)</t>
+      <t>(CB, WAS)</t>
     </r>
   </si>
   <si>
@@ -800,19 +887,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Jonnu Smith </t>
+      <t> Matthew Stafford </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(TE, GB)</t>
+      <t>(QB, LAR)</t>
     </r>
   </si>
   <si>
@@ -823,19 +908,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Baker Mayfield </t>
+      <t> C.J. Stroud </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(QB, TB)</t>
+      <t>(QB, HOU)</t>
     </r>
   </si>
   <si>
@@ -846,19 +929,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Matthew Stafford </t>
+      <t> Lamar Jackson </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(QB, LAR)</t>
+      <t>(QB, BAL)</t>
     </r>
   </si>
   <si>
@@ -869,19 +950,17 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Sam Darnold </t>
+      <t> Dak Prescott </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(QB, SEA)</t>
+      <t>(QB, DAL)</t>
     </r>
   </si>
   <si>
@@ -892,23 +971,18 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> Za'Darius Smith </t>
+      <t> Patrick Mahomes </t>
     </r>
     <r>
       <rPr>
         <sz val="8.8000000000000007"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t>(DE, ATL)</t>
+      <t>(QB, KC)</t>
     </r>
-  </si>
-  <si>
-    <t>TRENDING PAGES</t>
   </si>
   <si>
     <r>
@@ -918,8 +992,7 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
       <t> NFL Transactions</t>
     </r>
@@ -932,10 +1005,9 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> 2027 Running Back Free Agents</t>
+      <t> 2026 Cornerback Free Agents</t>
     </r>
   </si>
   <si>
@@ -946,10 +1018,9 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> 2020 Baltimore Ravens Free Agents</t>
+      <t> 2026 Cornerback Free Agents</t>
     </r>
   </si>
   <si>
@@ -960,10 +1031,9 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> 2026 Philadelphia Eagles Punter Salary Rankings</t>
+      <t> 2026 Denver Broncos Tackle Salary Rankings</t>
     </r>
   </si>
   <si>
@@ -974,10 +1044,9 @@
       <rPr>
         <sz val="8"/>
         <color rgb="FF4B566B"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <rFont val="Roboto"/>
       </rPr>
-      <t> NFL Agents</t>
+      <t> Guard Contra</t>
     </r>
   </si>
 </sst>
@@ -988,7 +1057,7 @@
   <numFmts count="1">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1101,12 +1170,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF4B566B"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF222222"/>
@@ -1114,22 +1177,46 @@
     </font>
     <font>
       <sz val="8"/>
+      <color rgb="FF4B566B"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <color rgb="FF373F50"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="4"/>
+      <color rgb="FF373F50"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF6C7C9B"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF373F50"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <color rgb="FF990000"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color rgb="FFCC3333"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <sz val="8.8000000000000007"/>
       <color rgb="FF4B566B"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Roboto"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1247,7 +1334,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1369,22 +1456,67 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="21" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="20" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="21" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="21" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
@@ -1411,14 +1543,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>6350</xdr:rowOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1456,11 +1588,56 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1026" name="AutoShape 2" descr="Podcast image">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6DD8E087-81B0-21BF-C695-CD94300DEACC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="7829550"/>
+          <a:ext cx="5715000" cy="5715000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1760,1073 +1937,1073 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5E8639F-25DA-4F52-8066-4D45988E24A4}">
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="44" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D1" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="E1" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="F1" s="24" t="s">
-        <v>98</v>
-      </c>
-      <c r="G1" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="H1" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="J1" s="22" t="s">
-        <v>94</v>
+      <c r="C1" s="44" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="45" t="s">
+        <v>104</v>
+      </c>
+      <c r="E1" s="45" t="s">
+        <v>105</v>
+      </c>
+      <c r="F1" s="45" t="s">
+        <v>106</v>
+      </c>
+      <c r="G1" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="H1" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="I1" s="45" t="s">
+        <v>109</v>
+      </c>
+      <c r="J1" s="45" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="25">
+      <c r="A2" s="47">
         <v>1</v>
       </c>
       <c r="B2" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="29">
-        <v>90</v>
-      </c>
-      <c r="D2" s="29">
+      <c r="C2" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2" s="48">
+        <v>53</v>
+      </c>
+      <c r="E2" s="48">
         <v>27.2</v>
       </c>
-      <c r="E2" s="30">
-        <v>261123758</v>
-      </c>
-      <c r="F2" s="31">
-        <v>80046766</v>
-      </c>
-      <c r="G2" s="30">
-        <v>313197111</v>
-      </c>
-      <c r="H2" s="30">
-        <v>27973413</v>
-      </c>
-      <c r="I2" s="30">
-        <v>261961018</v>
-      </c>
-      <c r="J2" s="30">
-        <v>36817740</v>
+      <c r="F2" s="49">
+        <v>287153511</v>
+      </c>
+      <c r="G2" s="50">
+        <v>54017013</v>
+      </c>
+      <c r="H2" s="49">
+        <v>215598105</v>
+      </c>
+      <c r="I2" s="49">
+        <v>19379933</v>
+      </c>
+      <c r="J2" s="49">
+        <v>41102783</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="27">
+      <c r="A3" s="51">
         <v>2</v>
       </c>
       <c r="B3" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="32">
-        <v>90</v>
-      </c>
-      <c r="D3" s="32">
+      <c r="C3" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="52">
+        <v>53</v>
+      </c>
+      <c r="E3" s="52">
         <v>26.3</v>
       </c>
-      <c r="E3" s="33">
-        <v>297438170</v>
-      </c>
-      <c r="F3" s="34">
-        <v>46279808</v>
-      </c>
-      <c r="G3" s="33">
-        <v>339610874</v>
-      </c>
-      <c r="H3" s="33">
-        <v>4107104</v>
-      </c>
-      <c r="I3" s="33">
-        <v>306576940</v>
-      </c>
-      <c r="J3" s="33">
-        <v>28406230</v>
+      <c r="F3" s="53">
+        <v>310081574</v>
+      </c>
+      <c r="G3" s="54">
+        <v>33636404</v>
+      </c>
+      <c r="H3" s="53">
+        <v>261541507</v>
+      </c>
+      <c r="I3" s="53">
+        <v>9042704</v>
+      </c>
+      <c r="J3" s="53">
+        <v>35206163</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="25">
+      <c r="A4" s="47">
         <v>3</v>
       </c>
       <c r="B4" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="29">
-        <v>90</v>
-      </c>
-      <c r="D4" s="29">
-        <v>26</v>
-      </c>
-      <c r="E4" s="30">
-        <v>261589836</v>
-      </c>
-      <c r="F4" s="31">
-        <v>44304649</v>
-      </c>
-      <c r="G4" s="30">
-        <v>302279836</v>
-      </c>
-      <c r="H4" s="30">
-        <v>3614649</v>
-      </c>
-      <c r="I4" s="30">
-        <v>291304986</v>
-      </c>
-      <c r="J4" s="30">
-        <v>5589850</v>
+      <c r="C4" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" s="48">
+        <v>53</v>
+      </c>
+      <c r="E4" s="48">
+        <v>26.8</v>
+      </c>
+      <c r="F4" s="49">
+        <v>273805454</v>
+      </c>
+      <c r="G4" s="50">
+        <v>32089031</v>
+      </c>
+      <c r="H4" s="49">
+        <v>253272548</v>
+      </c>
+      <c r="I4" s="49">
+        <v>8555381</v>
+      </c>
+      <c r="J4" s="49">
+        <v>7934725</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="27">
+      <c r="A5" s="51">
         <v>4</v>
       </c>
       <c r="B5" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="32">
-        <v>90</v>
-      </c>
-      <c r="D5" s="32">
-        <v>27.5</v>
-      </c>
-      <c r="E5" s="33">
-        <v>288406552</v>
-      </c>
-      <c r="F5" s="34">
-        <v>40224074</v>
-      </c>
-      <c r="G5" s="33">
-        <v>329692385</v>
-      </c>
-      <c r="H5" s="33">
-        <v>-1061759</v>
-      </c>
-      <c r="I5" s="33">
-        <v>304158821</v>
-      </c>
-      <c r="J5" s="33">
-        <v>22902731</v>
+      <c r="C5" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="52">
+        <v>53</v>
+      </c>
+      <c r="E5" s="52">
+        <v>27.3</v>
+      </c>
+      <c r="F5" s="53">
+        <v>303475221</v>
+      </c>
+      <c r="G5" s="54">
+        <v>25155405</v>
+      </c>
+      <c r="H5" s="53">
+        <v>241711046</v>
+      </c>
+      <c r="I5" s="53">
+        <v>33681985</v>
+      </c>
+      <c r="J5" s="53">
+        <v>24782790</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="25">
+      <c r="A6" s="47">
         <v>5</v>
       </c>
       <c r="B6" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="C6" s="29">
-        <v>89</v>
-      </c>
-      <c r="D6" s="29">
-        <v>26.5</v>
-      </c>
-      <c r="E6" s="30">
-        <v>266527994</v>
-      </c>
-      <c r="F6" s="31">
-        <v>37693906</v>
-      </c>
-      <c r="G6" s="30">
-        <v>305116564</v>
-      </c>
-      <c r="H6" s="30">
-        <v>-894664</v>
-      </c>
-      <c r="I6" s="30">
-        <v>298834072</v>
-      </c>
-      <c r="J6" s="30">
-        <v>3513922</v>
+      <c r="C6" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" s="48">
+        <v>53</v>
+      </c>
+      <c r="E6" s="48">
+        <v>27.2</v>
+      </c>
+      <c r="F6" s="49">
+        <v>280266697</v>
+      </c>
+      <c r="G6" s="50">
+        <v>23955203</v>
+      </c>
+      <c r="H6" s="49">
+        <v>258340275</v>
+      </c>
+      <c r="I6" s="49">
+        <v>11106480</v>
+      </c>
+      <c r="J6" s="49">
+        <v>6275156</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="27">
+      <c r="A7" s="51">
         <v>6</v>
       </c>
       <c r="B7" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="32">
-        <v>90</v>
-      </c>
-      <c r="D7" s="32">
-        <v>26.6</v>
-      </c>
-      <c r="E7" s="33">
-        <v>270012807</v>
-      </c>
-      <c r="F7" s="34">
-        <v>35599710</v>
-      </c>
-      <c r="G7" s="33">
-        <v>314824406</v>
-      </c>
-      <c r="H7" s="33">
-        <v>-9211889</v>
-      </c>
-      <c r="I7" s="33">
-        <v>263778370</v>
-      </c>
-      <c r="J7" s="33">
-        <v>44009437</v>
+      <c r="C7" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="52">
+        <v>53</v>
+      </c>
+      <c r="E7" s="52">
+        <v>27.3</v>
+      </c>
+      <c r="F7" s="53">
+        <v>283552429</v>
+      </c>
+      <c r="G7" s="54">
+        <v>22060088</v>
+      </c>
+      <c r="H7" s="53">
+        <v>219819960</v>
+      </c>
+      <c r="I7" s="53">
+        <v>12728469</v>
+      </c>
+      <c r="J7" s="53">
+        <v>46960300</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="25">
+      <c r="A8" s="47">
         <v>7</v>
       </c>
       <c r="B8" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="29">
-        <v>89</v>
-      </c>
-      <c r="D8" s="29">
-        <v>26</v>
-      </c>
-      <c r="E8" s="30">
-        <v>318003442</v>
-      </c>
-      <c r="F8" s="31">
-        <v>34975812</v>
-      </c>
-      <c r="G8" s="30">
-        <v>359076775</v>
-      </c>
-      <c r="H8" s="30">
-        <v>-6097521</v>
-      </c>
-      <c r="I8" s="30">
-        <v>314434128</v>
-      </c>
-      <c r="J8" s="30">
-        <v>38639314</v>
+      <c r="C8" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" s="48">
+        <v>53</v>
+      </c>
+      <c r="E8" s="48">
+        <v>26.1</v>
+      </c>
+      <c r="F8" s="49">
+        <v>332394856</v>
+      </c>
+      <c r="G8" s="50">
+        <v>20584398</v>
+      </c>
+      <c r="H8" s="49">
+        <v>260297586</v>
+      </c>
+      <c r="I8" s="49">
+        <v>26073944</v>
+      </c>
+      <c r="J8" s="49">
+        <v>42641126</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="27">
+      <c r="A9" s="51">
         <v>8</v>
       </c>
       <c r="B9" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="52">
+        <v>53</v>
+      </c>
+      <c r="E9" s="52">
+        <v>26.8</v>
+      </c>
+      <c r="F9" s="53">
+        <v>310223106</v>
+      </c>
+      <c r="G9" s="54">
+        <v>17884726</v>
+      </c>
+      <c r="H9" s="53">
+        <v>209488640</v>
+      </c>
+      <c r="I9" s="53">
+        <v>15876339</v>
+      </c>
+      <c r="J9" s="53">
+        <v>80898127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="47">
+        <v>9</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="48">
+        <v>53</v>
+      </c>
+      <c r="E10" s="48">
+        <v>27.4</v>
+      </c>
+      <c r="F10" s="49">
+        <v>304197291</v>
+      </c>
+      <c r="G10" s="50">
+        <v>17562781</v>
+      </c>
+      <c r="H10" s="49">
+        <v>272415499</v>
+      </c>
+      <c r="I10" s="49">
+        <v>9540882</v>
+      </c>
+      <c r="J10" s="49">
+        <v>18776810</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="51">
+        <v>10</v>
+      </c>
+      <c r="B11" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="52">
+        <v>53</v>
+      </c>
+      <c r="E11" s="52">
+        <v>26.3</v>
+      </c>
+      <c r="F11" s="53">
+        <v>297627260</v>
+      </c>
+      <c r="G11" s="54">
+        <v>17276671</v>
+      </c>
+      <c r="H11" s="53">
+        <v>205117262</v>
+      </c>
+      <c r="I11" s="53">
+        <v>41162301</v>
+      </c>
+      <c r="J11" s="53">
+        <v>47881797</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="47">
+        <v>11</v>
+      </c>
+      <c r="B12" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="32">
-        <v>88</v>
-      </c>
-      <c r="D9" s="32">
-        <v>25.6</v>
-      </c>
-      <c r="E9" s="33">
-        <v>305644001</v>
-      </c>
-      <c r="F9" s="34">
-        <v>33510201</v>
-      </c>
-      <c r="G9" s="33">
-        <v>352510978</v>
-      </c>
-      <c r="H9" s="33">
-        <v>-13356776</v>
-      </c>
-      <c r="I9" s="33">
-        <v>222795673</v>
-      </c>
-      <c r="J9" s="33">
-        <v>117153328</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="25">
-        <v>9</v>
-      </c>
-      <c r="B10" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="29">
-        <v>91</v>
-      </c>
-      <c r="D10" s="29">
-        <v>25.9</v>
-      </c>
-      <c r="E10" s="30">
-        <v>286462808</v>
-      </c>
-      <c r="F10" s="31">
-        <v>28441123</v>
-      </c>
-      <c r="G10" s="30">
-        <v>324422808</v>
-      </c>
-      <c r="H10" s="30">
-        <v>-9518877</v>
-      </c>
-      <c r="I10" s="30">
-        <v>276961366</v>
-      </c>
-      <c r="J10" s="30">
-        <v>45546442</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="27">
-        <v>10</v>
-      </c>
-      <c r="B11" s="28" t="s">
+      <c r="C12" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="48">
+        <v>53</v>
+      </c>
+      <c r="E12" s="48">
+        <v>25.7</v>
+      </c>
+      <c r="F12" s="49">
+        <v>324255917</v>
+      </c>
+      <c r="G12" s="50">
+        <v>14898285</v>
+      </c>
+      <c r="H12" s="49">
+        <v>188005389</v>
+      </c>
+      <c r="I12" s="49">
+        <v>14760059</v>
+      </c>
+      <c r="J12" s="49">
+        <v>118849869</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="51">
+        <v>12</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="52">
+        <v>53</v>
+      </c>
+      <c r="E13" s="52">
+        <v>27</v>
+      </c>
+      <c r="F13" s="53">
+        <v>300334638</v>
+      </c>
+      <c r="G13" s="54">
+        <v>14718624</v>
+      </c>
+      <c r="H13" s="53">
+        <v>283176480</v>
+      </c>
+      <c r="I13" s="53">
+        <v>10346190</v>
+      </c>
+      <c r="J13" s="53">
+        <v>2273268</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="47">
+        <v>13</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D14" s="48">
+        <v>53</v>
+      </c>
+      <c r="E14" s="48">
+        <v>26.6</v>
+      </c>
+      <c r="F14" s="49">
+        <v>289303460</v>
+      </c>
+      <c r="G14" s="50">
+        <v>14462170</v>
+      </c>
+      <c r="H14" s="49">
+        <v>259898239</v>
+      </c>
+      <c r="I14" s="49">
+        <v>5238758</v>
+      </c>
+      <c r="J14" s="49">
+        <v>19546763</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="51">
+        <v>14</v>
+      </c>
+      <c r="B15" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D15" s="52">
+        <v>53</v>
+      </c>
+      <c r="E15" s="52">
+        <v>26.9</v>
+      </c>
+      <c r="F15" s="53">
+        <v>305076411</v>
+      </c>
+      <c r="G15" s="54">
+        <v>12882502</v>
+      </c>
+      <c r="H15" s="53">
+        <v>289087963</v>
+      </c>
+      <c r="I15" s="53">
+        <v>1169130</v>
+      </c>
+      <c r="J15" s="53">
+        <v>11931218</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="47">
+        <v>15</v>
+      </c>
+      <c r="B16" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="C11" s="32">
-        <v>90</v>
-      </c>
-      <c r="D11" s="32">
-        <v>25.9</v>
-      </c>
-      <c r="E11" s="33">
-        <v>295557657</v>
-      </c>
-      <c r="F11" s="34">
-        <v>28306143</v>
-      </c>
-      <c r="G11" s="33">
-        <v>333937657</v>
-      </c>
-      <c r="H11" s="33">
-        <v>-10073857</v>
-      </c>
-      <c r="I11" s="33">
-        <v>220519457</v>
-      </c>
-      <c r="J11" s="33">
-        <v>111473200</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="25">
-        <v>11</v>
-      </c>
-      <c r="B12" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="29">
-        <v>90</v>
-      </c>
-      <c r="D12" s="29">
-        <v>26.2</v>
-      </c>
-      <c r="E12" s="30">
-        <v>276212456</v>
-      </c>
-      <c r="F12" s="31">
-        <v>27553174</v>
-      </c>
-      <c r="G12" s="30">
-        <v>314830789</v>
-      </c>
-      <c r="H12" s="30">
-        <v>-11065159</v>
-      </c>
-      <c r="I12" s="30">
-        <v>296469646</v>
-      </c>
-      <c r="J12" s="30">
-        <v>15737810</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="27">
-        <v>12</v>
-      </c>
-      <c r="B13" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="C13" s="32">
-        <v>90</v>
-      </c>
-      <c r="D13" s="32">
-        <v>26.7</v>
-      </c>
-      <c r="E13" s="33">
-        <v>285527736</v>
-      </c>
-      <c r="F13" s="34">
-        <v>25216623</v>
-      </c>
-      <c r="G13" s="33">
-        <v>330569664</v>
-      </c>
-      <c r="H13" s="33">
-        <v>-19825305</v>
-      </c>
-      <c r="I13" s="33">
-        <v>256924412</v>
-      </c>
-      <c r="J13" s="33">
-        <v>66758324</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="27">
-        <v>13</v>
-      </c>
-      <c r="B14" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14" s="32">
-        <v>89</v>
-      </c>
-      <c r="D14" s="32">
-        <v>26</v>
-      </c>
-      <c r="E14" s="33">
-        <v>292658959</v>
-      </c>
-      <c r="F14" s="34">
-        <v>22271338</v>
-      </c>
-      <c r="G14" s="33">
-        <v>330881125</v>
-      </c>
-      <c r="H14" s="33">
-        <v>-15950828</v>
-      </c>
-      <c r="I14" s="33">
-        <v>281655637</v>
-      </c>
-      <c r="J14" s="33">
-        <v>45473322</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="25">
-        <v>14</v>
-      </c>
-      <c r="B15" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" s="29">
-        <v>89</v>
-      </c>
-      <c r="D15" s="29">
-        <v>26.5</v>
-      </c>
-      <c r="E15" s="30">
-        <v>292881861</v>
-      </c>
-      <c r="F15" s="31">
-        <v>22171401</v>
-      </c>
-      <c r="G15" s="30">
-        <v>334732364</v>
-      </c>
-      <c r="H15" s="30">
-        <v>-19679102</v>
-      </c>
-      <c r="I15" s="30">
-        <v>327775425</v>
-      </c>
-      <c r="J15" s="30">
-        <v>596436</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="27">
-        <v>15</v>
-      </c>
-      <c r="B16" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" s="32">
-        <v>90</v>
-      </c>
-      <c r="D16" s="32">
-        <v>26.9</v>
-      </c>
-      <c r="E16" s="33">
-        <v>300205044</v>
-      </c>
-      <c r="F16" s="34">
-        <v>21555028</v>
-      </c>
-      <c r="G16" s="33">
-        <v>339745062</v>
-      </c>
-      <c r="H16" s="33">
-        <v>-17984990</v>
-      </c>
-      <c r="I16" s="33">
-        <v>324259598</v>
-      </c>
-      <c r="J16" s="33">
-        <v>12440446</v>
+      <c r="C16" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D16" s="48">
+        <v>53</v>
+      </c>
+      <c r="E16" s="48">
+        <v>26.3</v>
+      </c>
+      <c r="F16" s="49">
+        <v>311262220</v>
+      </c>
+      <c r="G16" s="50">
+        <v>12601580</v>
+      </c>
+      <c r="H16" s="49">
+        <v>186799412</v>
+      </c>
+      <c r="I16" s="49">
+        <v>5690390</v>
+      </c>
+      <c r="J16" s="49">
+        <v>114319218</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="25">
+      <c r="A17" s="47">
         <v>16</v>
       </c>
       <c r="B17" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="29">
-        <v>90</v>
-      </c>
-      <c r="D17" s="29">
-        <v>26.3</v>
-      </c>
-      <c r="E17" s="30">
-        <v>295696972</v>
-      </c>
-      <c r="F17" s="31">
-        <v>20926486</v>
-      </c>
-      <c r="G17" s="30">
-        <v>335946346</v>
-      </c>
-      <c r="H17" s="30">
-        <v>-19322888</v>
-      </c>
-      <c r="I17" s="30">
-        <v>258122552</v>
-      </c>
-      <c r="J17" s="30">
-        <v>74234420</v>
+      <c r="C17" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D17" s="48">
+        <v>53</v>
+      </c>
+      <c r="E17" s="48">
+        <v>26.7</v>
+      </c>
+      <c r="F17" s="49">
+        <v>305056946</v>
+      </c>
+      <c r="G17" s="50">
+        <v>11566512</v>
+      </c>
+      <c r="H17" s="49">
+        <v>221371256</v>
+      </c>
+      <c r="I17" s="49">
+        <v>5171752</v>
+      </c>
+      <c r="J17" s="49">
+        <v>75130838</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="27">
+      <c r="A18" s="51">
         <v>17</v>
       </c>
       <c r="B18" s="28" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="32">
-        <v>90</v>
-      </c>
-      <c r="D18" s="32">
-        <v>26.2</v>
-      </c>
-      <c r="E18" s="33">
-        <v>297581414</v>
-      </c>
-      <c r="F18" s="34">
-        <v>19934960</v>
-      </c>
-      <c r="G18" s="33">
-        <v>335604747</v>
-      </c>
-      <c r="H18" s="33">
-        <v>-18088373</v>
-      </c>
-      <c r="I18" s="33">
-        <v>320183827</v>
-      </c>
-      <c r="J18" s="33">
-        <v>13492587</v>
+      <c r="C18" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D18" s="52">
+        <v>53</v>
+      </c>
+      <c r="E18" s="52">
+        <v>26.6</v>
+      </c>
+      <c r="F18" s="53">
+        <v>307698424</v>
+      </c>
+      <c r="G18" s="54">
+        <v>9817950</v>
+      </c>
+      <c r="H18" s="53">
+        <v>283527751</v>
+      </c>
+      <c r="I18" s="53">
+        <v>4434426</v>
+      </c>
+      <c r="J18" s="53">
+        <v>15529647</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="25">
+      <c r="A19" s="47">
         <v>18</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="C19" s="29">
-        <v>88</v>
-      </c>
-      <c r="D19" s="29">
+        <v>62</v>
+      </c>
+      <c r="C19" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D19" s="48">
+        <v>53</v>
+      </c>
+      <c r="E19" s="48">
+        <v>25.3</v>
+      </c>
+      <c r="F19" s="49">
+        <v>299179988</v>
+      </c>
+      <c r="G19" s="50">
+        <v>9698455</v>
+      </c>
+      <c r="H19" s="49">
+        <v>104353562</v>
+      </c>
+      <c r="I19" s="49">
+        <v>9764828</v>
+      </c>
+      <c r="J19" s="49">
+        <v>182751298</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="51">
+        <v>19</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D20" s="52">
+        <v>54</v>
+      </c>
+      <c r="E20" s="52">
         <v>26.5</v>
       </c>
-      <c r="E19" s="30">
-        <v>300572901</v>
-      </c>
-      <c r="F19" s="31">
-        <v>17386012</v>
-      </c>
-      <c r="G19" s="30">
-        <v>335917901</v>
-      </c>
-      <c r="H19" s="30">
-        <v>-17958988</v>
-      </c>
-      <c r="I19" s="30">
-        <v>324989490</v>
-      </c>
-      <c r="J19" s="30">
-        <v>10928411</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="27">
-        <v>19</v>
-      </c>
-      <c r="B20" s="28" t="s">
+      <c r="F20" s="53">
+        <v>301822461</v>
+      </c>
+      <c r="G20" s="54">
+        <v>8921898</v>
+      </c>
+      <c r="H20" s="53">
+        <v>210076062</v>
+      </c>
+      <c r="I20" s="53">
+        <v>18277562</v>
+      </c>
+      <c r="J20" s="53">
+        <v>70499737</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="47">
+        <v>20</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" s="48">
+        <v>53</v>
+      </c>
+      <c r="E21" s="48">
+        <v>26.6</v>
+      </c>
+      <c r="F21" s="49">
+        <v>307084925</v>
+      </c>
+      <c r="G21" s="50">
+        <v>7845372</v>
+      </c>
+      <c r="H21" s="49">
+        <v>246796921</v>
+      </c>
+      <c r="I21" s="49">
+        <v>7190184</v>
+      </c>
+      <c r="J21" s="49">
+        <v>49221520</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="51">
+        <v>21</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="C22" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="52">
+        <v>53</v>
+      </c>
+      <c r="E22" s="52">
+        <v>27.3</v>
+      </c>
+      <c r="F22" s="53">
+        <v>307690215</v>
+      </c>
+      <c r="G22" s="54">
+        <v>6632908</v>
+      </c>
+      <c r="H22" s="53">
+        <v>286113128</v>
+      </c>
+      <c r="I22" s="53">
+        <v>5132176</v>
+      </c>
+      <c r="J22" s="53">
+        <v>11989011</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="47">
+        <v>22</v>
+      </c>
+      <c r="B23" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="C20" s="32">
-        <v>89</v>
-      </c>
-      <c r="D20" s="32">
-        <v>26.2</v>
-      </c>
-      <c r="E20" s="33">
-        <v>297700798</v>
-      </c>
-      <c r="F20" s="34">
-        <v>17025344</v>
-      </c>
-      <c r="G20" s="33">
-        <v>336910798</v>
-      </c>
-      <c r="H20" s="33">
-        <v>-22184656</v>
-      </c>
-      <c r="I20" s="33">
-        <v>313835417</v>
-      </c>
-      <c r="J20" s="33">
-        <v>18215381</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="25">
-        <v>20</v>
-      </c>
-      <c r="B21" s="26" t="s">
-        <v>96</v>
-      </c>
-      <c r="C21" s="29">
-        <v>89</v>
-      </c>
-      <c r="D21" s="29">
-        <v>26.5</v>
-      </c>
-      <c r="E21" s="30">
-        <v>297659015</v>
-      </c>
-      <c r="F21" s="31">
-        <v>16664108</v>
-      </c>
-      <c r="G21" s="30">
-        <v>336104015</v>
-      </c>
-      <c r="H21" s="30">
-        <v>-21780892</v>
-      </c>
-      <c r="I21" s="30">
-        <v>321490635</v>
-      </c>
-      <c r="J21" s="30">
-        <v>11568380</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="27">
-        <v>21</v>
-      </c>
-      <c r="B22" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="C22" s="32">
-        <v>90</v>
-      </c>
-      <c r="D22" s="32">
-        <v>25.4</v>
-      </c>
-      <c r="E22" s="33">
-        <v>292692188</v>
-      </c>
-      <c r="F22" s="34">
-        <v>16186255</v>
-      </c>
-      <c r="G22" s="33">
-        <v>330132188</v>
-      </c>
-      <c r="H22" s="33">
-        <v>-21253745</v>
-      </c>
-      <c r="I22" s="33">
-        <v>148588671</v>
-      </c>
-      <c r="J22" s="33">
-        <v>179888517</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="25">
-        <v>22</v>
-      </c>
-      <c r="B23" s="26" t="s">
+      <c r="C23" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" s="48">
+        <v>53</v>
+      </c>
+      <c r="E23" s="48">
+        <v>26.7</v>
+      </c>
+      <c r="F23" s="49">
+        <v>308248647</v>
+      </c>
+      <c r="G23" s="50">
+        <v>6477495</v>
+      </c>
+      <c r="H23" s="49">
+        <v>280061522</v>
+      </c>
+      <c r="I23" s="49">
+        <v>5087059</v>
+      </c>
+      <c r="J23" s="49">
+        <v>18887554</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="51">
+        <v>23</v>
+      </c>
+      <c r="B24" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="29">
-        <v>90</v>
-      </c>
-      <c r="D23" s="29">
+      <c r="C24" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="52">
+        <v>53</v>
+      </c>
+      <c r="E24" s="52">
+        <v>26.8</v>
+      </c>
+      <c r="F24" s="53">
+        <v>327114012</v>
+      </c>
+      <c r="G24" s="54">
+        <v>4951559</v>
+      </c>
+      <c r="H24" s="53">
+        <v>272831644</v>
+      </c>
+      <c r="I24" s="53">
+        <v>5249009</v>
+      </c>
+      <c r="J24" s="53">
+        <v>45567459</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="47">
+        <v>24</v>
+      </c>
+      <c r="B25" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" s="48">
+        <v>53</v>
+      </c>
+      <c r="E25" s="48">
         <v>26.3</v>
       </c>
-      <c r="E23" s="30">
-        <v>316008913</v>
-      </c>
-      <c r="F23" s="31">
-        <v>16056658</v>
-      </c>
-      <c r="G23" s="30">
-        <v>357208079</v>
-      </c>
-      <c r="H23" s="30">
-        <v>-25142508</v>
-      </c>
-      <c r="I23" s="30">
-        <v>311509591</v>
-      </c>
-      <c r="J23" s="30">
-        <v>42494322</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="27">
-        <v>23</v>
-      </c>
-      <c r="B24" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="C24" s="32">
-        <v>89</v>
-      </c>
-      <c r="D24" s="32">
+      <c r="F25" s="49">
+        <v>306312001</v>
+      </c>
+      <c r="G25" s="50">
+        <v>4401789</v>
+      </c>
+      <c r="H25" s="49">
+        <v>230940043</v>
+      </c>
+      <c r="I25" s="49">
+        <v>11135760</v>
+      </c>
+      <c r="J25" s="49">
+        <v>60030498</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="51">
+        <v>25</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D26" s="52">
+        <v>53</v>
+      </c>
+      <c r="E26" s="52">
+        <v>26.4</v>
+      </c>
+      <c r="F26" s="53">
+        <v>311027530</v>
+      </c>
+      <c r="G26" s="54">
+        <v>4174515</v>
+      </c>
+      <c r="H26" s="53">
+        <v>242673035</v>
+      </c>
+      <c r="I26" s="53">
+        <v>6194075</v>
+      </c>
+      <c r="J26" s="53">
+        <v>57788220</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="47">
+        <v>26</v>
+      </c>
+      <c r="B27" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D27" s="48">
+        <v>53</v>
+      </c>
+      <c r="E27" s="48">
         <v>26.6</v>
       </c>
-      <c r="E24" s="33">
-        <v>285420956</v>
-      </c>
-      <c r="F24" s="34">
-        <v>15395220</v>
-      </c>
-      <c r="G24" s="33">
-        <v>335345122</v>
-      </c>
-      <c r="H24" s="33">
-        <v>-34528946</v>
-      </c>
-      <c r="I24" s="33">
-        <v>295855041</v>
-      </c>
-      <c r="J24" s="33">
-        <v>27385915</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="25">
-        <v>24</v>
-      </c>
-      <c r="B25" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="C25" s="29">
-        <v>90</v>
-      </c>
-      <c r="D25" s="29">
-        <v>26.2</v>
-      </c>
-      <c r="E25" s="30">
-        <v>302963838</v>
-      </c>
-      <c r="F25" s="31">
-        <v>14808354</v>
-      </c>
-      <c r="G25" s="30">
-        <v>350436451</v>
-      </c>
-      <c r="H25" s="30">
-        <v>-32664259</v>
-      </c>
-      <c r="I25" s="30">
-        <v>225911622</v>
-      </c>
-      <c r="J25" s="30">
-        <v>114167216</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="27">
-        <v>25</v>
-      </c>
-      <c r="B26" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="C26" s="32">
-        <v>91</v>
-      </c>
-      <c r="D26" s="32">
-        <v>26.4</v>
-      </c>
-      <c r="E26" s="33">
-        <v>313629012</v>
-      </c>
-      <c r="F26" s="34">
-        <v>14478820</v>
-      </c>
-      <c r="G26" s="33">
-        <v>362736597</v>
-      </c>
-      <c r="H26" s="33">
-        <v>-34628765</v>
-      </c>
-      <c r="I26" s="33">
-        <v>279368191</v>
-      </c>
-      <c r="J26" s="33">
-        <v>73320820</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="25">
-        <v>26</v>
-      </c>
-      <c r="B27" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="C27" s="29">
-        <v>88</v>
-      </c>
-      <c r="D27" s="29">
-        <v>26.2</v>
-      </c>
-      <c r="E27" s="30">
-        <v>300960618</v>
-      </c>
-      <c r="F27" s="31">
-        <v>14241427</v>
-      </c>
-      <c r="G27" s="30">
-        <v>340693950</v>
-      </c>
-      <c r="H27" s="30">
-        <v>-25491905</v>
-      </c>
-      <c r="I27" s="30">
-        <v>279500898</v>
-      </c>
-      <c r="J27" s="30">
-        <v>56514720</v>
+      <c r="F27" s="49">
+        <v>300751799</v>
+      </c>
+      <c r="G27" s="50">
+        <v>829113</v>
+      </c>
+      <c r="H27" s="49">
+        <v>245232872</v>
+      </c>
+      <c r="I27" s="49">
+        <v>3434930</v>
+      </c>
+      <c r="J27" s="49">
+        <v>47207837</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="27">
+      <c r="A28" s="51">
         <v>27</v>
       </c>
       <c r="B28" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="32">
-        <v>90</v>
-      </c>
-      <c r="D28" s="32">
-        <v>26.3</v>
-      </c>
-      <c r="E28" s="33">
-        <v>310591393</v>
-      </c>
-      <c r="F28" s="34">
-        <v>12440706</v>
-      </c>
-      <c r="G28" s="33">
-        <v>349966427</v>
-      </c>
-      <c r="H28" s="33">
-        <v>-26934328</v>
-      </c>
-      <c r="I28" s="33">
-        <v>313163055</v>
-      </c>
-      <c r="J28" s="33">
-        <v>33848338</v>
+      <c r="C28" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D28" s="52">
+        <v>53</v>
+      </c>
+      <c r="E28" s="52">
+        <v>26.2</v>
+      </c>
+      <c r="F28" s="53">
+        <v>322247644</v>
+      </c>
+      <c r="G28" s="54">
+        <v>784455</v>
+      </c>
+      <c r="H28" s="53">
+        <v>265338463</v>
+      </c>
+      <c r="I28" s="53">
+        <v>17945144</v>
+      </c>
+      <c r="J28" s="53">
+        <v>35167837</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="25">
+      <c r="A29" s="47">
         <v>28</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>85</v>
-      </c>
-      <c r="C29" s="29">
-        <v>89</v>
-      </c>
-      <c r="D29" s="29">
-        <v>26.4</v>
-      </c>
-      <c r="E29" s="30">
-        <v>290733442</v>
-      </c>
-      <c r="F29" s="31">
-        <v>10847470</v>
-      </c>
-      <c r="G29" s="30">
-        <v>329633197</v>
-      </c>
-      <c r="H29" s="30">
-        <v>-28052285</v>
-      </c>
-      <c r="I29" s="30">
-        <v>280788897</v>
-      </c>
-      <c r="J29" s="30">
-        <v>46263711</v>
+        <v>83</v>
+      </c>
+      <c r="C29" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D29" s="48">
+        <v>53</v>
+      </c>
+      <c r="E29" s="48">
+        <v>26.7</v>
+      </c>
+      <c r="F29" s="49">
+        <v>301332434</v>
+      </c>
+      <c r="G29" s="50">
+        <v>-516258</v>
+      </c>
+      <c r="H29" s="49">
+        <v>257144531</v>
+      </c>
+      <c r="I29" s="49">
+        <v>11759166</v>
+      </c>
+      <c r="J29" s="49">
+        <v>28881837</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="27">
+      <c r="A30" s="51">
         <v>29</v>
       </c>
       <c r="B30" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="C30" s="32">
-        <v>90</v>
-      </c>
-      <c r="D30" s="32">
-        <v>26.3</v>
-      </c>
-      <c r="E30" s="33">
-        <v>302227469</v>
-      </c>
-      <c r="F30" s="34">
-        <v>10337202</v>
-      </c>
-      <c r="G30" s="33">
-        <v>344212761</v>
-      </c>
-      <c r="H30" s="33">
-        <v>-31648090</v>
-      </c>
-      <c r="I30" s="33">
-        <v>317658959</v>
-      </c>
-      <c r="J30" s="33">
-        <v>22253510</v>
+      <c r="C30" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D30" s="52">
+        <v>53</v>
+      </c>
+      <c r="E30" s="52">
+        <v>26.6</v>
+      </c>
+      <c r="F30" s="53">
+        <v>315684352</v>
+      </c>
+      <c r="G30" s="54">
+        <v>-3119681</v>
+      </c>
+      <c r="H30" s="53">
+        <v>224988626</v>
+      </c>
+      <c r="I30" s="53">
+        <v>62622717</v>
+      </c>
+      <c r="J30" s="53">
+        <v>24690809</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="25">
+      <c r="A31" s="47">
         <v>30</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="C31" s="29">
-        <v>90</v>
-      </c>
-      <c r="D31" s="29">
-        <v>26.2</v>
-      </c>
-      <c r="E31" s="30">
-        <v>302378394</v>
-      </c>
-      <c r="F31" s="31">
-        <v>8335396</v>
-      </c>
-      <c r="G31" s="30">
-        <v>341386092</v>
-      </c>
-      <c r="H31" s="30">
-        <v>-30672302</v>
-      </c>
-      <c r="I31" s="30">
-        <v>284065187</v>
-      </c>
-      <c r="J31" s="30">
-        <v>54858207</v>
+        <v>82</v>
+      </c>
+      <c r="C31" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D31" s="48">
+        <v>53</v>
+      </c>
+      <c r="E31" s="48">
+        <v>26.8</v>
+      </c>
+      <c r="F31" s="49">
+        <v>323611051</v>
+      </c>
+      <c r="G31" s="50">
+        <v>-5838859</v>
+      </c>
+      <c r="H31" s="49">
+        <v>182405091</v>
+      </c>
+      <c r="I31" s="49">
+        <v>20786614</v>
+      </c>
+      <c r="J31" s="49">
+        <v>117283746</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="27">
+      <c r="A32" s="51">
         <v>31</v>
       </c>
       <c r="B32" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D32" s="52">
+        <v>53</v>
+      </c>
+      <c r="E32" s="52">
+        <v>26.1</v>
+      </c>
+      <c r="F32" s="53">
+        <v>310014752</v>
+      </c>
+      <c r="G32" s="54">
+        <v>-7904003</v>
+      </c>
+      <c r="H32" s="53">
+        <v>285611049</v>
+      </c>
+      <c r="I32" s="53">
+        <v>5896448</v>
+      </c>
+      <c r="J32" s="53">
+        <v>15207855</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" s="55">
+        <v>32</v>
+      </c>
+      <c r="B33" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="C32" s="32">
-        <v>90</v>
-      </c>
-      <c r="D32" s="32">
-        <v>26.5</v>
-      </c>
-      <c r="E32" s="33">
-        <v>305047488</v>
-      </c>
-      <c r="F32" s="34">
-        <v>4867220</v>
-      </c>
-      <c r="G32" s="33">
-        <v>346254463</v>
-      </c>
-      <c r="H32" s="33">
-        <v>-36339755</v>
-      </c>
-      <c r="I32" s="33">
-        <v>322445499</v>
-      </c>
-      <c r="J32" s="33">
-        <v>20286989</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A33" s="35">
-        <v>32</v>
-      </c>
-      <c r="B33" s="36" t="s">
-        <v>77</v>
-      </c>
-      <c r="C33" s="37">
-        <v>90</v>
-      </c>
-      <c r="D33" s="37">
-        <v>25.7</v>
-      </c>
-      <c r="E33" s="38">
-        <v>298013269</v>
-      </c>
-      <c r="F33" s="39">
-        <v>4097480</v>
-      </c>
-      <c r="G33" s="38">
-        <v>336688268</v>
-      </c>
-      <c r="H33" s="38">
-        <v>-34577519</v>
-      </c>
-      <c r="I33" s="38">
-        <v>323279062</v>
-      </c>
-      <c r="J33" s="38">
-        <v>10279207</v>
+      <c r="C33" s="55" t="s">
+        <v>111</v>
+      </c>
+      <c r="D33" s="56">
+        <v>53</v>
+      </c>
+      <c r="E33" s="56">
+        <v>26.7</v>
+      </c>
+      <c r="F33" s="57">
+        <v>321669778</v>
+      </c>
+      <c r="G33" s="58">
+        <v>-11755070</v>
+      </c>
+      <c r="H33" s="57">
+        <v>273541723</v>
+      </c>
+      <c r="I33" s="57">
+        <v>22332308</v>
+      </c>
+      <c r="J33" s="57">
+        <v>22580047</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A34" s="42"/>
+      <c r="A34" s="40"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A35" s="43"/>
+      <c r="A35" s="42"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A36" s="40"/>
+      <c r="A36" s="59"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="40"/>
@@ -2915,165 +3092,168 @@
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" s="40"/>
     </row>
-    <row r="66" spans="1:1" ht="145" x14ac:dyDescent="0.35">
-      <c r="A66" s="44" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" s="40"/>
+    </row>
+    <row r="67" spans="1:1" ht="145" x14ac:dyDescent="0.35">
+      <c r="A67" s="43" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" s="40"/>
-    </row>
-    <row r="68" spans="1:1" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A68" s="44" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" s="40"/>
+    </row>
+    <row r="69" spans="1:1" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A69" s="43" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="69" spans="1:1" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A69" s="41" t="s">
+    <row r="70" spans="1:1" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A70" s="41" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="70" spans="1:1" ht="53.5" x14ac:dyDescent="0.35">
-      <c r="A70" s="45" t="s">
+    <row r="71" spans="1:1" ht="45" x14ac:dyDescent="0.35">
+      <c r="A71" s="60" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A72" s="61" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A73" s="61" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" ht="57.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A74" s="61" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="56" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A75" s="61" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A76" s="61" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A77" s="61" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A78" s="61" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" ht="56" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A79" s="61" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" ht="56" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A80" s="61" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="56" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A81" s="61" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A82" s="61" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" ht="56" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A83" s="61" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A84" s="61" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" ht="56" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A85" s="61" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A86" s="41" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="71" spans="1:1" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A71" s="46" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" ht="54" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A72" s="46" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" ht="54" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A73" s="46" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A74" s="46" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A75" s="46" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A76" s="46" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" ht="54" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A77" s="46" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A78" s="46" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" ht="54" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A79" s="46" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" ht="55.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A80" s="46" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" ht="54" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A81" s="46" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" ht="54" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A82" s="46" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A83" s="46" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" ht="55.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A84" s="46" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A85" s="41" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1" ht="30.5" x14ac:dyDescent="0.35">
-      <c r="A86" s="45" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" ht="51" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A87" s="46" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" ht="61" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A88" s="46" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" ht="81" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A89" s="46" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" ht="21" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A90" s="46" t="s">
-        <v>122</v>
+    <row r="87" spans="1:1" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="A87" s="60" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" ht="53" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A88" s="61" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="53" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A89" s="61" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A90" s="61" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" ht="21.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A91" s="61" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://www.spotrac.com/redirect/team/27/cap/2026" xr:uid="{1A811D61-272C-46DC-8FC8-BFBAC09A4004}"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://www.spotrac.com/redirect/team/16/cap/2026" xr:uid="{80C580E9-EA15-4C09-8A33-1DF01CD9F492}"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://www.spotrac.com/redirect/team/301/cap/2026" xr:uid="{E87B5972-86B0-4E56-A220-FD807820E67A}"/>
-    <hyperlink ref="B5" r:id="rId4" display="https://www.spotrac.com/redirect/team/973/cap/2026" xr:uid="{BE3B0BED-78EC-4020-9C76-82551D53C353}"/>
-    <hyperlink ref="B6" r:id="rId5" display="https://www.spotrac.com/redirect/team/9/cap/2026" xr:uid="{B85435FE-9354-4842-B0DC-38437CCEA5F7}"/>
-    <hyperlink ref="B7" r:id="rId6" display="https://www.spotrac.com/redirect/team/2/cap/2026" xr:uid="{0591E7D6-40B4-4432-B37A-5157BEEE4C56}"/>
-    <hyperlink ref="B8" r:id="rId7" display="https://www.spotrac.com/redirect/team/21/cap/2026" xr:uid="{665C69BD-8EF8-4A89-A4E8-58A9E647CF62}"/>
-    <hyperlink ref="B9" r:id="rId8" display="https://www.spotrac.com/redirect/team/7/cap/2026" xr:uid="{9066D488-7474-4817-8305-431C4C41EB13}"/>
-    <hyperlink ref="B10" r:id="rId9" display="https://www.spotrac.com/redirect/team/11/cap/2026" xr:uid="{B1155659-4DBB-4460-BF3E-9C4A051726FD}"/>
-    <hyperlink ref="B11" r:id="rId10" display="https://www.spotrac.com/redirect/team/24/cap/2026" xr:uid="{28583B64-06DA-494F-B1D1-69B8AF53A39D}"/>
-    <hyperlink ref="B12" r:id="rId11" display="https://www.spotrac.com/redirect/team/13/cap/2026" xr:uid="{21A08028-FC0D-4550-B5F8-4B86439A72A5}"/>
-    <hyperlink ref="B13" r:id="rId12" display="https://www.spotrac.com/redirect/team/12/cap/2026" xr:uid="{48C39884-4ABB-4F37-9D76-55BF6CE4B45A}"/>
-    <hyperlink ref="B14" r:id="rId13" display="https://www.spotrac.com/redirect/team/20/cap/2026" xr:uid="{FA3CEDBE-6A8D-4A02-A36A-92DB10EAA61F}"/>
-    <hyperlink ref="B15" r:id="rId14" display="https://www.spotrac.com/redirect/team/28/cap/2026" xr:uid="{534D0EDB-50FB-4FE9-B1B1-EEDD2615E251}"/>
-    <hyperlink ref="B16" r:id="rId15" display="https://www.spotrac.com/redirect/team/18/cap/2026" xr:uid="{EA3D4237-739F-4687-A929-61B9F3AE2F8B}"/>
-    <hyperlink ref="B17" r:id="rId16" display="https://www.spotrac.com/redirect/team/25/cap/2026" xr:uid="{0EEFC544-E5D2-41C4-A8FA-3B04B898A1B1}"/>
-    <hyperlink ref="B18" r:id="rId17" display="https://www.spotrac.com/redirect/team/30/cap/2026" xr:uid="{96C015B6-B606-44D6-B3AA-F6ED7278A532}"/>
-    <hyperlink ref="B19" r:id="rId18" display="https://www.spotrac.com/redirect/team/6/cap/2026" xr:uid="{32B50B75-4E5B-4CD2-89EA-F4B232ADF029}"/>
-    <hyperlink ref="B20" r:id="rId19" display="https://www.spotrac.com/redirect/team/3/cap/2026" xr:uid="{633E1F06-B316-4310-A431-4B6FDC38764E}"/>
-    <hyperlink ref="B21" r:id="rId20" display="https://www.spotrac.com/redirect/team/290/cap/2026" xr:uid="{54FBBB8C-F308-4E64-AA54-0E06071439F5}"/>
-    <hyperlink ref="B22" r:id="rId21" display="https://www.spotrac.com/redirect/team/19/cap/2026" xr:uid="{56CEBF4A-6CE3-46CA-94B0-E410B5F55C57}"/>
-    <hyperlink ref="B23" r:id="rId22" display="https://www.spotrac.com/redirect/team/8/cap/2026" xr:uid="{A9A4BD84-6703-4FEC-9625-DEBAEC4C2E46}"/>
-    <hyperlink ref="B24" r:id="rId23" display="https://www.spotrac.com/redirect/team/23/cap/2026" xr:uid="{57847E6A-6D59-4AAB-A709-4C037FF78053}"/>
-    <hyperlink ref="B25" r:id="rId24" display="https://www.spotrac.com/redirect/team/22/cap/2026" xr:uid="{D1C343CC-B8FE-4B9C-BC20-8A01332DC9B6}"/>
-    <hyperlink ref="B26" r:id="rId25" display="https://www.spotrac.com/redirect/team/1/cap/2026" xr:uid="{1196ADAF-E803-4AC0-B891-9ED98653F928}"/>
-    <hyperlink ref="B27" r:id="rId26" display="https://www.spotrac.com/redirect/team/367/cap/2026" xr:uid="{A9CAD66D-32DC-4AE2-BD66-1C3A8FBCF7DB}"/>
-    <hyperlink ref="B28" r:id="rId27" display="https://www.spotrac.com/redirect/team/10/cap/2026" xr:uid="{ACFDB361-EDD6-41B3-AF5A-3835CDEB2EAD}"/>
-    <hyperlink ref="B29" r:id="rId28" display="https://www.spotrac.com/redirect/team/62/cap/2026" xr:uid="{B2BD90F0-E996-4B88-8180-AD7B5E5307A5}"/>
-    <hyperlink ref="B30" r:id="rId29" display="https://www.spotrac.com/redirect/team/4/cap/2026" xr:uid="{8641781D-1DA8-4BD1-8283-3C7BEE2C2AAC}"/>
-    <hyperlink ref="B31" r:id="rId30" display="https://www.spotrac.com/redirect/team/14/cap/2026" xr:uid="{2667352F-81C1-4ED2-B660-121A8F47D5A8}"/>
-    <hyperlink ref="B32" r:id="rId31" display="https://www.spotrac.com/redirect/team/5/cap/2026" xr:uid="{B19CF7BE-1D68-4A56-937D-966D995167A4}"/>
-    <hyperlink ref="B33" r:id="rId32" display="https://www.spotrac.com/redirect/team/15/cap/2026" xr:uid="{056017FE-BDC1-4923-BE1E-85A781B602C8}"/>
-    <hyperlink ref="A66" r:id="rId33" display="https://www.spotrac.com/podcasts/_/id/3446/deshaun-watson-james-harden-the-expiring-contract-nfl-fantasy-draft" xr:uid="{2991B619-5F8A-41E7-8608-F23521AFA142}"/>
-    <hyperlink ref="A68" r:id="rId34" display="https://www.spotrac.com/podcasts/_/id/3446/deshaun-watson-james-harden-the-expiring-contract-nfl-fantasy-draft" xr:uid="{8C5632B3-79E4-408F-B9D7-43C17ADD4A5E}"/>
+    <hyperlink ref="B2" r:id="rId1" display="https://www.spotrac.com/redirect/team/27/cap/2026" xr:uid="{35A50113-8A05-4E8A-BF52-F1D0A709E03C}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://www.spotrac.com/redirect/team/16/cap/2026" xr:uid="{3C8FAA36-3D80-4D6E-B060-D31E77E712C3}"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://www.spotrac.com/redirect/team/301/cap/2026" xr:uid="{C68F6060-02E5-471E-BE49-27A6061EFD31}"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://www.spotrac.com/redirect/team/973/cap/2026" xr:uid="{99B17B68-A1AB-4A7C-8C27-2F3CFC316295}"/>
+    <hyperlink ref="B6" r:id="rId5" display="https://www.spotrac.com/redirect/team/9/cap/2026" xr:uid="{DE33E4B9-6067-4B6D-8377-1EC78D550918}"/>
+    <hyperlink ref="B7" r:id="rId6" display="https://www.spotrac.com/redirect/team/2/cap/2026" xr:uid="{F4B1EA00-417A-478B-890C-EA6884ADCCB3}"/>
+    <hyperlink ref="B8" r:id="rId7" display="https://www.spotrac.com/redirect/team/21/cap/2026" xr:uid="{861D84A4-7758-4CC9-B736-AF1AB3E5A013}"/>
+    <hyperlink ref="B9" r:id="rId8" display="https://www.spotrac.com/redirect/team/1/cap/2026" xr:uid="{A8131E26-54F2-48A6-BDA8-841CC0C02ADD}"/>
+    <hyperlink ref="B10" r:id="rId9" display="https://www.spotrac.com/redirect/team/18/cap/2026" xr:uid="{6658C0D5-962E-4A72-8461-EADE01E24E46}"/>
+    <hyperlink ref="B11" r:id="rId10" display="https://www.spotrac.com/redirect/team/11/cap/2026" xr:uid="{D3EE65E0-92B6-4916-B65D-DD417C104222}"/>
+    <hyperlink ref="B12" r:id="rId11" display="https://www.spotrac.com/redirect/team/7/cap/2026" xr:uid="{7CA41938-5CF9-49D7-90C8-6DB46B2A3411}"/>
+    <hyperlink ref="B13" r:id="rId12" display="https://www.spotrac.com/redirect/team/28/cap/2026" xr:uid="{DFC55736-EDF3-4EB2-A740-A06D422E0B00}"/>
+    <hyperlink ref="B14" r:id="rId13" display="https://www.spotrac.com/redirect/team/13/cap/2026" xr:uid="{C2396FB9-AE43-47C6-B337-D8B77AF8059F}"/>
+    <hyperlink ref="B15" r:id="rId14" display="https://www.spotrac.com/redirect/team/6/cap/2026" xr:uid="{9C5B6829-F08A-41C8-ADFA-4523896CE37C}"/>
+    <hyperlink ref="B16" r:id="rId15" display="https://www.spotrac.com/redirect/team/24/cap/2026" xr:uid="{69B153C2-E815-49AA-ABE1-30F7EE75A360}"/>
+    <hyperlink ref="B17" r:id="rId16" display="https://www.spotrac.com/redirect/team/25/cap/2026" xr:uid="{65763F15-3469-4435-8C4D-44C396A3464D}"/>
+    <hyperlink ref="B18" r:id="rId17" display="https://www.spotrac.com/redirect/team/30/cap/2026" xr:uid="{C66F5D42-EEF0-4E46-BF08-95767BDFCF0A}"/>
+    <hyperlink ref="B19" r:id="rId18" display="https://www.spotrac.com/redirect/team/19/cap/2026" xr:uid="{0A3219C0-1866-4D50-A984-A6CEB02AD63E}"/>
+    <hyperlink ref="B20" r:id="rId19" display="https://www.spotrac.com/redirect/team/12/cap/2026" xr:uid="{E0AFF6F7-B86F-49E2-B13E-9FEF4433D74F}"/>
+    <hyperlink ref="B21" r:id="rId20" display="https://www.spotrac.com/redirect/team/20/cap/2026" xr:uid="{EA7FDE02-DC3F-490F-AD95-DE504FE78AB9}"/>
+    <hyperlink ref="B22" r:id="rId21" display="https://www.spotrac.com/redirect/team/290/cap/2026" xr:uid="{2FC5A8C2-AD88-4789-BE99-5CE5580BEA10}"/>
+    <hyperlink ref="B23" r:id="rId22" display="https://www.spotrac.com/redirect/team/3/cap/2026" xr:uid="{635D7904-FD9D-4C12-AAB3-53E9BF8FE330}"/>
+    <hyperlink ref="B24" r:id="rId23" display="https://www.spotrac.com/redirect/team/8/cap/2026" xr:uid="{9F68D123-A608-4F8A-B7F8-F8F083E6D2D0}"/>
+    <hyperlink ref="B25" r:id="rId24" display="https://www.spotrac.com/redirect/team/14/cap/2026" xr:uid="{76EE00A1-5C16-4318-BC85-6767082624E2}"/>
+    <hyperlink ref="B26" r:id="rId25" display="https://www.spotrac.com/redirect/team/367/cap/2026" xr:uid="{D22B5C3B-87EB-4D9E-AF85-9E7FC7BC490C}"/>
+    <hyperlink ref="B27" r:id="rId26" display="https://www.spotrac.com/redirect/team/62/cap/2026" xr:uid="{60908F39-CE85-4172-804A-5F7E120B4639}"/>
+    <hyperlink ref="B28" r:id="rId27" display="https://www.spotrac.com/redirect/team/10/cap/2026" xr:uid="{67E61AC0-87D2-4084-9B97-23387E8A2E44}"/>
+    <hyperlink ref="B29" r:id="rId28" display="https://www.spotrac.com/redirect/team/23/cap/2026" xr:uid="{D8CA961C-5A27-41F7-9BA4-EB75B3E59DC2}"/>
+    <hyperlink ref="B30" r:id="rId29" display="https://www.spotrac.com/redirect/team/4/cap/2026" xr:uid="{3E48EAD2-2943-49A6-8DCC-1B2801B3EB66}"/>
+    <hyperlink ref="B31" r:id="rId30" display="https://www.spotrac.com/redirect/team/22/cap/2026" xr:uid="{F571DFBC-1EA5-4BCD-A27F-71C270807B30}"/>
+    <hyperlink ref="B32" r:id="rId31" display="https://www.spotrac.com/redirect/team/15/cap/2026" xr:uid="{66ECFA79-83BA-495C-B7A8-3F212633A18F}"/>
+    <hyperlink ref="B33" r:id="rId32" display="https://www.spotrac.com/redirect/team/5/cap/2026" xr:uid="{5DAD3776-4F11-48F6-A0B7-0E361E4871AE}"/>
+    <hyperlink ref="A67" r:id="rId33" display="https://www.spotrac.com/podcasts/_/id/3446/deshaun-watson-james-harden-the-expiring-contract-nfl-fantasy-draft" xr:uid="{4118CD64-411C-43E1-B31A-85E8B488C629}"/>
+    <hyperlink ref="A69" r:id="rId34" display="https://www.spotrac.com/podcasts/_/id/3446/deshaun-watson-james-harden-the-expiring-contract-nfl-fantasy-draft" xr:uid="{93B6999E-7EDD-483D-9741-7AC894BC3FB4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId35"/>

</xml_diff>